<commit_message>
Isler temasini bordo yap ve logoyu yaklastir
</commit_message>
<xml_diff>
--- a/output/Fiyat-Listesi-Yonetim.xlsx
+++ b/output/Fiyat-Listesi-Yonetim.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="Rb9dd5a23b66a45b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="R9262368db7854836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="R775ad0901e7e4d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="Rebb04810d08b444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="Rab84dffcb1dc4beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="Re1d4f43611cc4a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Rcb48a92fe6cc48f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="Rdbd497cab81f4766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="Rdeca6853128843f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="Ra0511d50af9c4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="R996a66dfab0c4b67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="R42e02c8ff9e94a68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="R666c7c55ba99497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Raf168619436e4b31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2506,79 +2506,58 @@
     <x:t xml:space="preserve">Dosya GitHub'a yüklendiğinde web programı ve PDF otomatik yenilenir.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Sınıf Ayarları</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Kitabevi Listesi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Yayınevi - Kitabevi Eşleştirmesi</x:t>
+    <x:t xml:space="preserve">7</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Yeni bir yayınevi ekleyip Güncelle düğmesine bastığınızda Ayarlar listesine otomatik eklenir. Karşısındaki Kitabevi Kodu'nu seçin.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">8</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Logo göstermek için Sayfa Ayarları sayfasındaki Logo Linki alanına doğrudan görsel bağlantısını yapıştırın.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Kitabevi Kodu</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Kademe</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Kitabevi Kodu</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Kitabevi Adı</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Yayınevi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">5. Sınıf</x:t>
+    <x:t xml:space="preserve">Ad Soyad</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Telefon</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">WhatsApp</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">kitabevi-1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Ortaokul</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">kitabevi-1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">İşer Kitabevi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">6. Sınıf</x:t>
+    <x:t xml:space="preserve">Aytaç Arslan</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">5345556747</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Evet</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Emre Arslan</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">5466779329</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Lise</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">kitabevi-2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mega Kitabevi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">7. Sınıf</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">8. Sınıf</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Lise</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ad Soyad</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Telefon</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">WhatsApp</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Aytaç Arslan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">5345556747</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Evet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Emre Arslan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">5466779329</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Furkan ÖZKAN</x:t>
@@ -2646,7 +2625,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2701,11 +2680,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF2B134"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2797,7 +2771,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2920,13 +2894,16 @@
     <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2937,34 +2914,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -19060,60 +19009,60 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="Rf5868dd89b114609"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="R139e728302704965"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="R9d436fde78d847ef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="Rd8980e6915fa48fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="R19ede4a5d10448b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="Rd496114d2bd24d9a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="Reb1880f43a694ce6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="R9defe46981424341"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="R9f75206da06e41a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="R77e803aa1f114c17"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="R9aaa654bcb524a1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="R80e6cf0c9705469a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="R479e1e1130b64201"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R606d0612f771420f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="Rf74ddffd193e43e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="R37a87eba675940d3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="Rb76e57d610fe4af8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="Rddce47f265e24177"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="R535827b203c74fc6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="Rfe8781b183484799"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="R87c26f48771b475a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="Rd28f55383f4c43b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="R37766e3ab8be4e0b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="R338ae189e6ce4ebd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R05f3bb55c9d645f4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R220e00d5b2fd4343"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="Rcc7ba72105774d5d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rb92eaffb5fd84575"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R3737a0c6bc204ab3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="R251931cf7b114d91"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="R1dada3a02c224bf4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="R4fe669b275564fc2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R7af2151606ea480c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="R5b8c448ed9ed4f68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="R50796819c2ab4943"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="Rce65394aec5b4d3f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="Rd06211eecaef4aba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="R6376df39372c43ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R958d641523014cc4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="R850011debe614713"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="Rcc41b3dc65ff492f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="Rb50101c11e5c498e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="R674d6173b8b04fe2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="R7137ee80738b43e2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="Rb2d1fbbffb694e88"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="R677bf6eb7b3549a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R56a3c8d98b3d49d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="R15dac2b878e247b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R1b6983c0ad7044df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="Rb21da75fbbcf427e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="R9c25b7fc9ba04b8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="Rc35f41db43904b65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="R15121bc8272e4445"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="R0c4aa081762a4840"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="R5825bf036bd644b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="R35c1d17b51554f63"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="R5fb3e2c7e3b74b4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="Rd64f6c6552ff4c10"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="Rd1f517dbd2244ffb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="R261f4722a7264218"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="R32fb441d8b7f4376"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="R4e596ae772da4897"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="Re67af15ef7aa4095"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R112e8a82d4824799"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="R0c272d30add241ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="R273e02cb07274204"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="R778b73da12864683"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="R0fcad0137ab9416c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="R4a866e3d62de4129"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="R558cc9c3211d441d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="Rc3ded1653a17486b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="R785663d842604955"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="R6c79ac8360fd487d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="Rdd8e9707cebe4cf9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R163051eca9f54356"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R2d94d485b14f439a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="R410697465a0e4e64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rd9088c8f37f748a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R9203f6c6d0b046d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="Rfa3b8b79ec9a4b75"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="Rdeac31759a884340"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="Rf154bf395ca94dc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R6b62c2d289004d2e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="Rce60f66630004022"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="R91f1a572b9ab4139"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="R44371b6fd936426f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="Re45cc429d0744e83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="R3509699e1b0d4f34"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R0682b8e219104b05"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="Rb66d5e8f78b44cd9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="R4b546eb8f610442c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="Ra42efcc00050457b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="Rd79703fe22b042d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="R7a465e84a8b44926"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="R80ea31a41eb0494d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="Rae3473b411e94a88"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R5d81b9c3355b4725"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="Rd0399517eaa24661"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R20fcd5911be74c3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="R957a40037e7f41aa"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb561f65cb6f64d04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ca0f94852084e6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20677,7 +20626,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4d258532f4b4aec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ec948967a424468"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20739,19 +20688,19 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="82" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" customWidth="1"/>
+    <x:col min="2" max="2" width="82" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="51" t="s">
+      <x:c r="A1" s="52" t="s">
         <x:v>816</x:v>
       </x:c>
-      <x:c r="B1" s="51"/>
-      <x:c r="C1" s="51"/>
-      <x:c r="D1" s="51"/>
-      <x:c r="E1" s="51"/>
-      <x:c r="F1" s="51"/>
+      <x:c r="B1" s="52"/>
+      <x:c r="C1" s="52"/>
+      <x:c r="D1" s="52"/>
+      <x:c r="E1" s="52"/>
+      <x:c r="F1" s="52"/>
     </x:row>
     <x:row r="3" ht="33.95000076293945" customHeight="1">
       <x:c r="A3" s="26" t="s">
@@ -20807,20 +20756,20 @@
         <x:v>829</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="40" customHeight="1">
-      <x:c r="A10" s="27" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B10" s="27" t="str">
-        <x:v>Yeni bir yayınevi ekleyip Güncelle düğmesine bastığınızda Ayarlar listesine otomatik eklenir. Karşısındaki Kitabevi Kodu'nu seçin.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="40" customHeight="1">
-      <x:c r="A11" s="27" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B11" s="27" t="str">
-        <x:v>Logo göstermek için Sayfa Ayarları sayfasındaki Logo Linki alanına doğrudan görsel bağlantısını yapıştırın.</x:v>
+    <x:row r="10" ht="39.95000076293945" customHeight="1">
+      <x:c r="A10" s="27" t="s">
+        <x:v>830</x:v>
+      </x:c>
+      <x:c r="B10" s="27" t="s">
+        <x:v>831</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39.95000076293945" customHeight="1">
+      <x:c r="A11" s="27" t="s">
+        <x:v>832</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="s">
+        <x:v>833</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20843,389 +20792,542 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32.099998474121094" customHeight="1">
-      <x:c r="A1" s="52" t="s">
-        <x:v>830</x:v>
-      </x:c>
-      <x:c r="B1" s="52"/>
-      <x:c r="D1" s="52" t="s">
-        <x:v>831</x:v>
-      </x:c>
-      <x:c r="E1" s="52"/>
-      <x:c r="G1" s="53" t="s">
-        <x:v>832</x:v>
-      </x:c>
-      <x:c r="H1" s="53"/>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1"/>
+      <x:c r="A1" s="53" t="str">
+        <x:v>Sınıf Ayarları</x:v>
+      </x:c>
+      <x:c r="B1" s="53"/>
+      <x:c r="C1"/>
+      <x:c r="D1" s="53" t="str">
+        <x:v>Kitabevi Listesi</x:v>
+      </x:c>
+      <x:c r="E1" s="53"/>
+      <x:c r="F1"/>
+      <x:c r="G1" s="54" t="str">
+        <x:v>Yayınevi - Kitabevi Eşleştirmesi</x:v>
+      </x:c>
+      <x:c r="H1" s="54"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+    </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="32" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="32" t="s">
-        <x:v>833</x:v>
-      </x:c>
-      <x:c r="D3" s="32" t="s">
-        <x:v>834</x:v>
-      </x:c>
-      <x:c r="E3" s="32" t="s">
-        <x:v>835</x:v>
-      </x:c>
-      <x:c r="G3" s="47" t="s">
-        <x:v>836</x:v>
-      </x:c>
-      <x:c r="H3" s="47" t="s">
-        <x:v>834</x:v>
+      <x:c r="A3" s="32" t="str">
+        <x:v>Sınıf</x:v>
+      </x:c>
+      <x:c r="B3" s="32" t="str">
+        <x:v>Kademe</x:v>
+      </x:c>
+      <x:c r="C3"/>
+      <x:c r="D3" s="32" t="str">
+        <x:v>Kitabevi Kodu</x:v>
+      </x:c>
+      <x:c r="E3" s="32" t="str">
+        <x:v>Kitabevi Adı</x:v>
+      </x:c>
+      <x:c r="F3"/>
+      <x:c r="G3" s="47" t="str">
+        <x:v>Yayınevi</x:v>
+      </x:c>
+      <x:c r="H3" s="47" t="str">
+        <x:v>Kitabevi Kodu</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="33" t="s">
-        <x:v>837</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="s">
-        <x:v>838</x:v>
-      </x:c>
-      <x:c r="D4" s="36" t="s">
-        <x:v>839</x:v>
-      </x:c>
-      <x:c r="E4" s="36" t="s">
-        <x:v>840</x:v>
-      </x:c>
+      <x:c r="A4" s="33" t="str">
+        <x:v>5. Sınıf</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>Ortaokul</x:v>
+      </x:c>
+      <x:c r="C4"/>
+      <x:c r="D4" s="36" t="str">
+        <x:v>kitabevi-1</x:v>
+      </x:c>
+      <x:c r="E4" s="36" t="str">
+        <x:v>İşler Kitabevi</x:v>
+      </x:c>
+      <x:c r="F4"/>
       <x:c r="G4" s="3" t="str">
         <x:v>4K</x:v>
       </x:c>
-      <x:c r="H4" s="64" t="str">
+      <x:c r="H4" s="50" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="34" t="s">
-        <x:v>841</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="s">
-        <x:v>838</x:v>
-      </x:c>
-      <x:c r="D5" s="37" t="s">
-        <x:v>842</x:v>
-      </x:c>
-      <x:c r="E5" s="37" t="s">
-        <x:v>843</x:v>
-      </x:c>
+      <x:c r="A5" s="34" t="str">
+        <x:v>6. Sınıf</x:v>
+      </x:c>
+      <x:c r="B5" s="34" t="str">
+        <x:v>Ortaokul</x:v>
+      </x:c>
+      <x:c r="C5"/>
+      <x:c r="D5" s="37" t="str">
+        <x:v>kitabevi-2</x:v>
+      </x:c>
+      <x:c r="E5" s="37" t="str">
+        <x:v>Mega Kitabevi</x:v>
+      </x:c>
+      <x:c r="F5"/>
       <x:c r="G5" s="4" t="str">
         <x:v>Acil Yayınları</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="34" t="s">
-        <x:v>844</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="s">
-        <x:v>838</x:v>
-      </x:c>
+      <x:c r="A6" s="34" t="str">
+        <x:v>7. Sınıf</x:v>
+      </x:c>
+      <x:c r="B6" s="34" t="str">
+        <x:v>Ortaokul</x:v>
+      </x:c>
+      <x:c r="C6"/>
       <x:c r="D6" s="37"/>
       <x:c r="E6" s="37"/>
+      <x:c r="F6"/>
       <x:c r="G6" s="4" t="str">
         <x:v>Aktif Öğrenme Yayınları</x:v>
       </x:c>
-      <x:c r="H6" s="65" t="str">
+      <x:c r="H6" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="34" t="s">
-        <x:v>845</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="s">
-        <x:v>838</x:v>
-      </x:c>
+      <x:c r="A7" s="34" t="str">
+        <x:v>8. Sınıf</x:v>
+      </x:c>
+      <x:c r="B7" s="34" t="str">
+        <x:v>Ortaokul</x:v>
+      </x:c>
+      <x:c r="C7"/>
       <x:c r="D7" s="37"/>
       <x:c r="E7" s="37"/>
+      <x:c r="F7"/>
       <x:c r="G7" s="4" t="str">
         <x:v>Alan Yayınları</x:v>
       </x:c>
-      <x:c r="H7" s="65" t="str">
+      <x:c r="H7" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="34" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="s">
-        <x:v>846</x:v>
-      </x:c>
+      <x:c r="A8" s="34" t="str">
+        <x:v>9. Sınıf</x:v>
+      </x:c>
+      <x:c r="B8" s="34" t="str">
+        <x:v>Lise</x:v>
+      </x:c>
+      <x:c r="C8"/>
       <x:c r="D8" s="37"/>
       <x:c r="E8" s="37"/>
+      <x:c r="F8"/>
       <x:c r="G8" s="4" t="str">
         <x:v>Apotemi Yayınları</x:v>
       </x:c>
-      <x:c r="H8" s="65" t="str">
+      <x:c r="H8" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="34" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="B9" s="34" t="s">
-        <x:v>846</x:v>
-      </x:c>
+      <x:c r="A9" s="34" t="str">
+        <x:v>10. Sınıf</x:v>
+      </x:c>
+      <x:c r="B9" s="34" t="str">
+        <x:v>Lise</x:v>
+      </x:c>
+      <x:c r="C9"/>
       <x:c r="D9" s="37"/>
       <x:c r="E9" s="37"/>
+      <x:c r="F9"/>
       <x:c r="G9" s="4" t="str">
         <x:v>Aydın</x:v>
       </x:c>
-      <x:c r="H9" s="65" t="str">
+      <x:c r="H9" s="51" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="34" t="s">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="B10" s="34" t="s">
-        <x:v>846</x:v>
-      </x:c>
+      <x:c r="A10" s="34" t="str">
+        <x:v>11. Sınıf</x:v>
+      </x:c>
+      <x:c r="B10" s="34" t="str">
+        <x:v>Lise</x:v>
+      </x:c>
+      <x:c r="C10"/>
       <x:c r="D10" s="37"/>
       <x:c r="E10" s="37"/>
+      <x:c r="F10"/>
       <x:c r="G10" s="4" t="str">
         <x:v>Bilgi Arşivi Yayınları</x:v>
       </x:c>
-      <x:c r="H10" s="65" t="str">
+      <x:c r="H10" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="34" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="B11" s="34" t="s">
-        <x:v>846</x:v>
-      </x:c>
+      <x:c r="A11" s="34" t="str">
+        <x:v>12. Sınıf</x:v>
+      </x:c>
+      <x:c r="B11" s="34" t="str">
+        <x:v>Lise</x:v>
+      </x:c>
+      <x:c r="C11"/>
       <x:c r="D11" s="37"/>
       <x:c r="E11" s="37"/>
+      <x:c r="F11"/>
       <x:c r="G11" s="4" t="str">
         <x:v>Bilgi Sarmal Yayınları</x:v>
       </x:c>
-      <x:c r="H11" s="65" t="str">
+      <x:c r="H11" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="35" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B12" s="35" t="s">
-        <x:v>846</x:v>
-      </x:c>
+      <x:c r="A12" s="35" t="str">
+        <x:v>Maarif TYT</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Lise</x:v>
+      </x:c>
+      <x:c r="C12"/>
       <x:c r="D12" s="37"/>
       <x:c r="E12" s="37"/>
+      <x:c r="F12"/>
       <x:c r="G12" s="4" t="str">
         <x:v>Biyotik Yayınları</x:v>
       </x:c>
-      <x:c r="H12" s="65" t="str">
+      <x:c r="H12" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
       <x:c r="D13" s="37"/>
       <x:c r="E13" s="37"/>
+      <x:c r="F13"/>
       <x:c r="G13" s="4" t="str">
         <x:v>Coğrafya Gurmesi Yayınları</x:v>
       </x:c>
-      <x:c r="H13" s="65" t="str">
+      <x:c r="H13" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
       <x:c r="D14" s="37"/>
       <x:c r="E14" s="37"/>
+      <x:c r="F14"/>
       <x:c r="G14" s="4" t="str">
         <x:v>Çap Yayınları</x:v>
       </x:c>
-      <x:c r="H14" s="65" t="str">
+      <x:c r="H14" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
       <x:c r="D15" s="37"/>
       <x:c r="E15" s="37"/>
+      <x:c r="F15"/>
       <x:c r="G15" s="4" t="str">
         <x:v>Edebiyat Sokağı Yayınları</x:v>
       </x:c>
-      <x:c r="H15" s="65" t="str">
+      <x:c r="H15" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
       <x:c r="D16" s="37"/>
       <x:c r="E16" s="37"/>
+      <x:c r="F16"/>
       <x:c r="G16" s="4" t="str">
         <x:v>Egzersiz Yayınları</x:v>
       </x:c>
-      <x:c r="H16" s="65" t="str">
+      <x:c r="H16" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
       <x:c r="D17" s="37"/>
       <x:c r="E17" s="37"/>
+      <x:c r="F17"/>
       <x:c r="G17" s="4" t="str">
         <x:v>Eğitim Vadisi</x:v>
       </x:c>
-      <x:c r="H17" s="65" t="str">
+      <x:c r="H17" s="51" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
       <x:c r="D18" s="37"/>
       <x:c r="E18" s="37"/>
+      <x:c r="F18"/>
       <x:c r="G18" s="4" t="str">
         <x:v>ENS Yayınları</x:v>
       </x:c>
-      <x:c r="H18" s="65" t="str">
+      <x:c r="H18" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
       <x:c r="D19" s="37"/>
       <x:c r="E19" s="37"/>
+      <x:c r="F19"/>
       <x:c r="G19" s="4" t="str">
         <x:v>Etkili Matematik Yayınları</x:v>
       </x:c>
-      <x:c r="H19" s="65" t="str">
+      <x:c r="H19" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
       <x:c r="D20" s="38"/>
       <x:c r="E20" s="38"/>
+      <x:c r="F20"/>
       <x:c r="G20" s="4" t="str">
         <x:v>Fizik Pedia Yayınları</x:v>
       </x:c>
-      <x:c r="H20" s="65" t="str">
+      <x:c r="H20" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
       <x:c r="G21" s="4" t="str">
         <x:v>Full Matematik Yayınları</x:v>
       </x:c>
-      <x:c r="H21" s="65" t="str">
+      <x:c r="H21" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
       <x:c r="G22" s="4" t="str">
         <x:v>Hız ve Renk Yayınları</x:v>
       </x:c>
-      <x:c r="H22" s="65" t="str">
+      <x:c r="H22" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
       <x:c r="G23" s="4" t="str">
         <x:v>Limit</x:v>
       </x:c>
-      <x:c r="H23" s="65" t="str">
+      <x:c r="H23" s="51" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
       <x:c r="G24" s="4" t="str">
         <x:v>Mikro Orijinal Yayınları</x:v>
       </x:c>
-      <x:c r="H24" s="65" t="str">
+      <x:c r="H24" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
       <x:c r="G25" s="4" t="str">
         <x:v>Miray</x:v>
       </x:c>
-      <x:c r="H25" s="65" t="str">
+      <x:c r="H25" s="51" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
       <x:c r="G26" s="4" t="str">
         <x:v>Oktet Yayınları</x:v>
       </x:c>
-      <x:c r="H26" s="65" t="str">
+      <x:c r="H26" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
       <x:c r="G27" s="4" t="str">
         <x:v>Orbital Yayınları</x:v>
       </x:c>
-      <x:c r="H27" s="65" t="str">
+      <x:c r="H27" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
       <x:c r="G28" s="4" t="str">
         <x:v>Orijinal Matematik Yayınları</x:v>
       </x:c>
-      <x:c r="H28" s="65" t="str">
+      <x:c r="H28" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
       <x:c r="G29" s="4" t="str">
         <x:v>Profizik</x:v>
       </x:c>
-      <x:c r="H29" s="65" t="str">
+      <x:c r="H29" s="51" t="str">
         <x:v>kitabevi-2</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
       <x:c r="G30" s="4" t="str">
         <x:v>Rehber Matematik Yayınları</x:v>
       </x:c>
-      <x:c r="H30" s="65" t="str">
+      <x:c r="H30" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
       <x:c r="G31" s="4" t="str">
         <x:v>Ritim Biyoloji Yayınları</x:v>
       </x:c>
-      <x:c r="H31" s="65" t="str">
+      <x:c r="H31" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
       <x:c r="G32" s="4" t="str">
         <x:v>Süre Yayınları</x:v>
       </x:c>
-      <x:c r="H32" s="65" t="str">
+      <x:c r="H32" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
       <x:c r="G33" s="4" t="str">
         <x:v>Ulti Yayınları</x:v>
       </x:c>
-      <x:c r="H33" s="65" t="str">
+      <x:c r="H33" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
       <x:c r="G34" s="4" t="str">
         <x:v>Viral Yayınları</x:v>
       </x:c>
-      <x:c r="H34" s="65" t="str">
+      <x:c r="H34" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
+      <x:c r="E35"/>
+      <x:c r="F35"/>
       <x:c r="G35" s="4" t="str">
         <x:v>Yarıçap Yayınları</x:v>
       </x:c>
-      <x:c r="H35" s="65" t="str">
+      <x:c r="H35" s="51" t="str">
         <x:v>kitabevi-1</x:v>
       </x:c>
     </x:row>
@@ -21242,8 +21344,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4389774e21894828"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a07e837b7ed414a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R781cc4c197b74aa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15d5d0827bc0428c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21258,7 +21360,7 @@
     <x:col min="4" max="4" width="52" customWidth="1"/>
     <x:col min="5" max="6" width="16" customWidth="1"/>
     <x:col min="7" max="8" width="17" customWidth="1"/>
-    <x:col min="9" max="9" width="46" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="46" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -21286,7 +21388,7 @@
       <x:c r="H1" s="39" t="str">
         <x:v>Ana Sayfa Sırası</x:v>
       </x:c>
-      <x:c r="I1" s="57" t="str">
+      <x:c r="I1" s="48" t="str">
         <x:v>Logo Linki</x:v>
       </x:c>
     </x:row>
@@ -21302,7 +21404,7 @@
         <x:v>Ortaokul kitapları ve güncel fiyat listesi</x:v>
       </x:c>
       <x:c r="E2" s="40" t="str">
-        <x:v>#173F5F</x:v>
+        <x:v>#8B1E2D</x:v>
       </x:c>
       <x:c r="F2" s="40" t="str">
         <x:v>#F2B134</x:v>
@@ -21313,7 +21415,7 @@
       <x:c r="H2" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I2" s="60" t="str">
+      <x:c r="I2" s="49" t="str">
         <x:v>assets/logos/isler-kitabevi.png</x:v>
       </x:c>
     </x:row>
@@ -21329,7 +21431,7 @@
         <x:v>Lise kitapları ve güncel fiyat listesi</x:v>
       </x:c>
       <x:c r="E3" s="41" t="str">
-        <x:v>#173F5F</x:v>
+        <x:v>#8B1E2D</x:v>
       </x:c>
       <x:c r="F3" s="41" t="str">
         <x:v>#F2B134</x:v>
@@ -21340,7 +21442,7 @@
       <x:c r="H3" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I3" s="60" t="str">
+      <x:c r="I3" s="49" t="str">
         <x:v>assets/logos/isler-kitabevi.png</x:v>
       </x:c>
     </x:row>
@@ -21367,7 +21469,7 @@
       <x:c r="H4" s="41" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I4" s="60" t="str">
+      <x:c r="I4" s="49" t="str">
         <x:v>assets/logos/mega-kitabevi.png</x:v>
       </x:c>
     </x:row>
@@ -21394,7 +21496,7 @@
       <x:c r="H5" s="41" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I5" s="60" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>assets/logos/mega-kitabevi.png</x:v>
       </x:c>
     </x:row>
@@ -21559,7 +21661,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf46de4659a614dd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295d7b50697848cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21580,16 +21682,16 @@
         <x:v>834</x:v>
       </x:c>
       <x:c r="B1" s="43" t="s">
-        <x:v>833</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="C1" s="43" t="s">
-        <x:v>847</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="D1" s="43" t="s">
-        <x:v>848</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="E1" s="43" t="s">
-        <x:v>849</x:v>
+        <x:v>838</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.100000381469727" customHeight="1">
@@ -21597,16 +21699,16 @@
         <x:v>839</x:v>
       </x:c>
       <x:c r="B2" s="40" t="s">
-        <x:v>838</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="C2" s="40" t="s">
-        <x:v>850</x:v>
+        <x:v>841</x:v>
       </x:c>
       <x:c r="D2" s="44" t="s">
-        <x:v>851</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="E2" s="40" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.100000381469727" customHeight="1">
@@ -21614,16 +21716,16 @@
         <x:v>839</x:v>
       </x:c>
       <x:c r="B3" s="41" t="s">
-        <x:v>838</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="C3" s="41" t="s">
-        <x:v>853</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="D3" s="45" t="s">
-        <x:v>854</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="E3" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
@@ -21634,13 +21736,13 @@
         <x:v>846</x:v>
       </x:c>
       <x:c r="C4" s="40" t="s">
-        <x:v>850</x:v>
+        <x:v>841</x:v>
       </x:c>
       <x:c r="D4" s="44" t="s">
-        <x:v>851</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="E4" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.100000381469727" customHeight="1">
@@ -21651,65 +21753,65 @@
         <x:v>846</x:v>
       </x:c>
       <x:c r="C5" s="41" t="s">
-        <x:v>853</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="D5" s="45" t="s">
-        <x:v>854</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="E5" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.100000381469727" customHeight="1">
       <x:c r="A6" s="41" t="s">
-        <x:v>842</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B6" s="41" t="s">
-        <x:v>838</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="C6" s="41" t="s">
-        <x:v>855</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="D6" s="45" t="s">
-        <x:v>856</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="E6" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26.100000381469727" customHeight="1">
       <x:c r="A7" s="41" t="s">
-        <x:v>842</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B7" s="41" t="s">
-        <x:v>838</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="C7" s="41"/>
       <x:c r="D7" s="45"/>
       <x:c r="E7" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.100000381469727" customHeight="1">
       <x:c r="A8" s="41" t="s">
-        <x:v>842</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B8" s="41" t="s">
         <x:v>846</x:v>
       </x:c>
       <x:c r="C8" s="41" t="s">
-        <x:v>855</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="D8" s="45" t="s">
-        <x:v>856</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="E8" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.100000381469727" customHeight="1">
       <x:c r="A9" s="41" t="s">
-        <x:v>842</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B9" s="41" t="s">
         <x:v>846</x:v>
@@ -21717,7 +21819,7 @@
       <x:c r="C9" s="41"/>
       <x:c r="D9" s="45"/>
       <x:c r="E9" s="41" t="s">
-        <x:v>852</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26.100000381469727" customHeight="1">
@@ -21948,7 +22050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33d900a4f3514b2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb88dbe0dbf4696"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Mega temasini ve baslik gorunumunu guncelle
</commit_message>
<xml_diff>
--- a/output/Fiyat-Listesi-Yonetim.xlsx
+++ b/output/Fiyat-Listesi-Yonetim.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="Rdbd497cab81f4766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="Rdeca6853128843f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="Ra0511d50af9c4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="R996a66dfab0c4b67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="R42e02c8ff9e94a68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="R666c7c55ba99497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Raf168619436e4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="R3ae31ddbde894f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="R320adc1706574c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="R7663e8f2e5cf4a94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="R2bc3fb719c954739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="R71fc2aea5c764a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="R9ea8b890059247f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Rd9b6d26d5dd740c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19009,60 +19009,60 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="R9c25b7fc9ba04b8b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="Rc35f41db43904b65"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="R15121bc8272e4445"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="R0c4aa081762a4840"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="R5825bf036bd644b7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="R35c1d17b51554f63"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="R5fb3e2c7e3b74b4b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="Rd64f6c6552ff4c10"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="Rd1f517dbd2244ffb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="R261f4722a7264218"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="R32fb441d8b7f4376"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="R4e596ae772da4897"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="Re67af15ef7aa4095"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R112e8a82d4824799"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="R0c272d30add241ee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="R273e02cb07274204"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="R778b73da12864683"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="R0fcad0137ab9416c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="R4a866e3d62de4129"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="R558cc9c3211d441d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="Rc3ded1653a17486b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="R785663d842604955"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="R6c79ac8360fd487d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="Rdd8e9707cebe4cf9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R163051eca9f54356"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R2d94d485b14f439a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="R410697465a0e4e64"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rd9088c8f37f748a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R9203f6c6d0b046d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="Rfa3b8b79ec9a4b75"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="Rdeac31759a884340"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="Rf154bf395ca94dc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R6b62c2d289004d2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="Rce60f66630004022"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="R91f1a572b9ab4139"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="R44371b6fd936426f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="Re45cc429d0744e83"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="R3509699e1b0d4f34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R0682b8e219104b05"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="Rb66d5e8f78b44cd9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="R4b546eb8f610442c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="Ra42efcc00050457b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="Rd79703fe22b042d6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="R7a465e84a8b44926"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="R80ea31a41eb0494d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="Rae3473b411e94a88"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R5d81b9c3355b4725"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="Rd0399517eaa24661"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R20fcd5911be74c3c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="R957a40037e7f41aa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="Rd8fc043c275f4faa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="R2561cc4ee1594b65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="Rb2aceca866fa4fe8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="Rce6e3fe5f05b43dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="Rff7660c4bd644334"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="Rcb7ee03f6a3c413e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="Rff010bb958ac47c4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="R25104c90ea1f428a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="R67ccf0d21d77419c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="Rfa9ff748d62e4404"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="Rb3d05134ff0c41d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="R7cd52b9a4e404342"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="Re1e257ef89f947c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R088731e22c7d4c12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="Ra0316cd905e4447c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="R9697e3ad6c6d401b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="R238159b02fe84cd6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="R7e0c49203b244d64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="R936e89cb65e24a3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="R1e715b7fd5614bc5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="Rb34ce3853f214e21"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="Rfed8911ecd0a4a90"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="Ra6825685fab64d3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="R3e9d6edc76da4e5c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R36aa12ff38ee4b52"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R2a4c1e0ac032479f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="R30bba635fc6145ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rfe5dd124df124fc7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R0549a48388254140"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="Re3d0d94a50e34078"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="R1e49bcd5f91544b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="R0329512bb9544b59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R95ef9c7fa454440b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="R925cb52d62b64aad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="R065d3c25985b4c3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="Rc1b79a89a4b0488d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="R4c1bb36bfb6e4dd2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="Reabce9a2992c4025"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R4c08202f34934bef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="R9f835619f0674099"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="Rb6dd3e4394c544c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="R0a8534a3af414a65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="R06909328d0074b01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="Rfc8ae3dae2e44a10"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="R16949d0edaaf4d8c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="R5ff4137e468243e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R7989af1fc5bf4e95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="R3941217fbba64707"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R340e7b7de94e409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="R0f2c4c02059b40f8"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ca0f94852084e6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra64380c6a9834c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20626,7 +20626,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ec948967a424468"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b87a4137a1b4dcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21344,8 +21344,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R781cc4c197b74aa3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15d5d0827bc0428c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf18931f488434aef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R058eb3f5690348f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21458,10 +21458,10 @@
         <x:v>Ortaokul kitapları ve güncel fiyat listesi</x:v>
       </x:c>
       <x:c r="E4" s="41" t="str">
-        <x:v>#234E52</x:v>
+        <x:v>#211F20</x:v>
       </x:c>
       <x:c r="F4" s="41" t="str">
-        <x:v>#F6C453</x:v>
+        <x:v>#F6B500</x:v>
       </x:c>
       <x:c r="G4" s="41" t="str">
         <x:v>Evet</x:v>
@@ -21485,10 +21485,10 @@
         <x:v>Lise kitapları ve güncel fiyat listesi</x:v>
       </x:c>
       <x:c r="E5" s="41" t="str">
-        <x:v>#234E52</x:v>
+        <x:v>#211F20</x:v>
       </x:c>
       <x:c r="F5" s="41" t="str">
-        <x:v>#F6C453</x:v>
+        <x:v>#F6B500</x:v>
       </x:c>
       <x:c r="G5" s="41" t="str">
         <x:v>Evet</x:v>
@@ -21661,7 +21661,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295d7b50697848cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d1b5c0df7cf42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22050,7 +22050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb88dbe0dbf4696"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc827c749ae4f5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Kataloglar arasi gecis ayari ekle
</commit_message>
<xml_diff>
--- a/output/Fiyat-Listesi-Yonetim.xlsx
+++ b/output/Fiyat-Listesi-Yonetim.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="R3ae31ddbde894f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="R320adc1706574c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="R7663e8f2e5cf4a94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="R2bc3fb719c954739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="R71fc2aea5c764a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="R9ea8b890059247f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Rd9b6d26d5dd740c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünler" sheetId="1" r:id="R5da03a1f94064d93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İndirimler" sheetId="2" r:id="R280de119b2ef4dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasarım" sheetId="3" r:id="Re076a537326a4e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="4" r:id="Ra9b9c9a01a124e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ayarlar" sheetId="5" r:id="R5e2293e460704ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa Ayarları" sheetId="6" r:id="Rea7644fd068e40de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İletişim" sheetId="7" r:id="Ra3cbeeadadf34d3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2625,7 +2625,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2690,6 +2690,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173F5F"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2771,7 +2781,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2915,6 +2925,18 @@
     <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Köprü" xfId="1"/>
@@ -19009,60 +19031,60 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="Rd8fc043c275f4faa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="R2561cc4ee1594b65"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="Rb2aceca866fa4fe8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="Rce6e3fe5f05b43dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="Rff7660c4bd644334"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="Rcb7ee03f6a3c413e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="Rff010bb958ac47c4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="R25104c90ea1f428a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="R67ccf0d21d77419c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="Rfa9ff748d62e4404"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="Rb3d05134ff0c41d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="R7cd52b9a4e404342"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="Re1e257ef89f947c8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R088731e22c7d4c12"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="Ra0316cd905e4447c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="R9697e3ad6c6d401b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="R238159b02fe84cd6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="R7e0c49203b244d64"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="R936e89cb65e24a3c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="R1e715b7fd5614bc5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="Rb34ce3853f214e21"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="Rfed8911ecd0a4a90"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="Ra6825685fab64d3a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="R3e9d6edc76da4e5c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R36aa12ff38ee4b52"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R2a4c1e0ac032479f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="R30bba635fc6145ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rfe5dd124df124fc7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R0549a48388254140"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="Re3d0d94a50e34078"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="R1e49bcd5f91544b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="R0329512bb9544b59"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R95ef9c7fa454440b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="R925cb52d62b64aad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="R065d3c25985b4c3b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="Rc1b79a89a4b0488d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="R4c1bb36bfb6e4dd2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="Reabce9a2992c4025"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R4c08202f34934bef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="R9f835619f0674099"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="Rb6dd3e4394c544c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="R0a8534a3af414a65"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="R06909328d0074b01"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="Rfc8ae3dae2e44a10"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="R16949d0edaaf4d8c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="R5ff4137e468243e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R7989af1fc5bf4e95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="R3941217fbba64707"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R340e7b7de94e409a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="R0f2c4c02059b40f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="Ra8b67e8a81354fd7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="R8c5cf00ff194490e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="R725be37277c543f3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="Ra593d1ddc2fc4882"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="R6509f43898a04599"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="R215bf2246fd841bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="R4c04e84133a94f8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="Rbb2734d666d543df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="R9e50211ab0cb4730"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="R2e678d0f34bb4a1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="R8c76c90be3034c77"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="Ra2a6a84574f343f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="R24153d84382a41c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="R635ae4f039c9487f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="Redb89279cd0e485c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="Rdbb00d72b4c84839"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="Re83fc8638c124ce1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="Rd1ccfb348218407e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="Re0a6ea2c8e54482e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="Rf313729fe30e4795"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="R46ebd285693e4d75"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="Rba62afe623364400"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="R626d8dbed8eb40c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="R87d62b242cdc486e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="R4e548c3690be4ebc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="R6a04c76cbbc941e2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="R3c7123c9e44144bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="Rf73cd085d5ba43fd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="R8386705a60ca4889"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="R5e74deb9eea44f86"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="R9537430d9bca428d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="R8151916a3e244916"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="R0b2e0e1d5f104d82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="R5c6601b0895b41e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="Rb8a8df9a658947c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="Reb6a853e1e4742ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="R4d4bf19c2c5b4ca3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="R120c72a0715446ad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="R204f8e6cf97a46c5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="R689aae3ee0324e46"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="Re74a224ed1624358"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="R2f45e80e886d442b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="Rd28b7aede8f64e8c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="Rc56d741c5c964a2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="Rd14db475bb504c0d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J429" r:id="R1550de81fb724024"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J431" r:id="R993139d7d9184734"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J439" r:id="Re611f794205c4f87"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J458" r:id="R749489d8afa04074"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J470" r:id="Rc72dc4c170b94d2a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra64380c6a9834c43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb2340301db948f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20626,7 +20648,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b87a4137a1b4dcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd100b30ec8fc4ed8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21344,8 +21366,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf18931f488434aef"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R058eb3f5690348f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43b3f84bf12d4d25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa22a70df890427e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21361,6 +21383,7 @@
     <x:col min="5" max="6" width="16" customWidth="1"/>
     <x:col min="7" max="8" width="17" customWidth="1"/>
     <x:col min="9" max="9" width="46" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -21391,6 +21414,9 @@
       <x:c r="I1" s="48" t="str">
         <x:v>Logo Linki</x:v>
       </x:c>
+      <x:c r="J1" s="59" t="str">
+        <x:v>Gösterilecek Diğer Liste</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="40" t="str">
@@ -21418,6 +21444,9 @@
       <x:c r="I2" s="49" t="str">
         <x:v>assets/logos/isler-kitabevi.png</x:v>
       </x:c>
+      <x:c r="J2" s="60" t="str">
+        <x:v>kitabevi-2 | Ortaokul</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="41" t="str">
@@ -21445,6 +21474,9 @@
       <x:c r="I3" s="49" t="str">
         <x:v>assets/logos/isler-kitabevi.png</x:v>
       </x:c>
+      <x:c r="J3" s="60" t="str">
+        <x:v>kitabevi-2 | Lise</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="41" t="str">
@@ -21472,6 +21504,9 @@
       <x:c r="I4" s="49" t="str">
         <x:v>assets/logos/mega-kitabevi.png</x:v>
       </x:c>
+      <x:c r="J4" s="60" t="str">
+        <x:v>kitabevi-1 | Ortaokul</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="41" t="str">
@@ -21498,6 +21533,9 @@
       </x:c>
       <x:c r="I5" s="49" t="str">
         <x:v>assets/logos/mega-kitabevi.png</x:v>
+      </x:c>
+      <x:c r="J5" s="60" t="str">
+        <x:v>kitabevi-1 | Lise</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="27.950000762939453" customHeight="1">
@@ -21651,17 +21689,20 @@
       <x:c r="H20" s="42"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="G2:G20">
       <x:formula1>"Evet,Hayır"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B2:B20">
       <x:formula1>"Ortaokul,Lise"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="J2:J100">
+      <x:formula1>"Yok,kitabevi-1 | Ortaokul,kitabevi-1 | Lise,kitabevi-2 | Ortaokul,kitabevi-2 | Lise"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d1b5c0df7cf42ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8753ffe177cc4b7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22050,7 +22091,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc827c749ae4f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b37a75beed14015"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>